<commit_message>
Updated MEX model - 2025-11-25 01:08
</commit_message>
<xml_diff>
--- a/VerveStacks_MEX/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_MEX/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_MEX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800BF9F4-6463-47AE-A5F1-95071BAC9829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7044F8A-7A66-4EFF-9591-C95BB9CCD5B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="56" r:id="rId1"/>

</xml_diff>